<commit_message>
Extended smooth transitions beyond -20 and +60 degrees C.
</commit_message>
<xml_diff>
--- a/DOCUMENTS/TEMPERATURE-TO-COLOR-MAP.xlsx
+++ b/DOCUMENTS/TEMPERATURE-TO-COLOR-MAP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Andre\ENGINEERING\PROJECTS\MECHATRONIX LAB\ColorTemp\DOCUMENTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579EBA89-7C64-4FB3-868B-953C721AE357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA0C112-CF24-41F4-BF91-C74CE11C2563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C62921F5-4B94-4ED4-BA24-C9546B752848}"/>
+    <workbookView xWindow="14400" yWindow="-32400" windowWidth="29010" windowHeight="16305" xr2:uid="{C62921F5-4B94-4ED4-BA24-C9546B752848}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,6 +89,18 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -116,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -143,6 +155,15 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -222,263 +243,383 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$42</c:f>
+              <c:f>Sheet1!$A$2:$A$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
+                <c:ptCount val="61"/>
                 <c:pt idx="0">
+                  <c:v>-400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-380</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-360</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-340</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-320</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-300</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-280</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-260</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-240</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-220</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>-200</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="11">
                   <c:v>-180</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="12">
                   <c:v>-160</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="13">
                   <c:v>-140</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="14">
                   <c:v>-120</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="15">
                   <c:v>-100</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="16">
                   <c:v>-80</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="17">
                   <c:v>-60</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="18">
                   <c:v>-40</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="19">
                   <c:v>-20</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="22">
                   <c:v>40</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="23">
                   <c:v>60</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="24">
                   <c:v>80</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="25">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="26">
                   <c:v>120</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="27">
                   <c:v>140</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="28">
                   <c:v>160</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="29">
                   <c:v>180</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="30">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="31">
                   <c:v>220</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="32">
                   <c:v>240</c:v>
                 </c:pt>
-                <c:pt idx="23">
+                <c:pt idx="33">
                   <c:v>260</c:v>
                 </c:pt>
-                <c:pt idx="24">
+                <c:pt idx="34">
                   <c:v>280</c:v>
                 </c:pt>
-                <c:pt idx="25">
+                <c:pt idx="35">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="26">
+                <c:pt idx="36">
                   <c:v>320</c:v>
                 </c:pt>
-                <c:pt idx="27">
+                <c:pt idx="37">
                   <c:v>340</c:v>
                 </c:pt>
-                <c:pt idx="28">
+                <c:pt idx="38">
                   <c:v>360</c:v>
                 </c:pt>
-                <c:pt idx="29">
+                <c:pt idx="39">
                   <c:v>380</c:v>
                 </c:pt>
-                <c:pt idx="30">
+                <c:pt idx="40">
                   <c:v>400</c:v>
                 </c:pt>
-                <c:pt idx="31">
+                <c:pt idx="41">
                   <c:v>420</c:v>
                 </c:pt>
-                <c:pt idx="32">
+                <c:pt idx="42">
                   <c:v>440</c:v>
                 </c:pt>
-                <c:pt idx="33">
+                <c:pt idx="43">
                   <c:v>460</c:v>
                 </c:pt>
-                <c:pt idx="34">
+                <c:pt idx="44">
                   <c:v>480</c:v>
                 </c:pt>
-                <c:pt idx="35">
+                <c:pt idx="45">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="36">
+                <c:pt idx="46">
                   <c:v>520</c:v>
                 </c:pt>
-                <c:pt idx="37">
+                <c:pt idx="47">
                   <c:v>540</c:v>
                 </c:pt>
-                <c:pt idx="38">
+                <c:pt idx="48">
                   <c:v>560</c:v>
                 </c:pt>
-                <c:pt idx="39">
+                <c:pt idx="49">
                   <c:v>580</c:v>
                 </c:pt>
-                <c:pt idx="40">
+                <c:pt idx="50">
                   <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>620</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>640</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>660</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>680</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>720</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>740</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>760</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>780</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>800</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$42</c:f>
+              <c:f>Sheet1!$B$2:$B$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
+                <c:ptCount val="61"/>
                 <c:pt idx="0">
                   <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>900</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="12">
                   <c:v>800</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="13">
                   <c:v>700</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="14">
                   <c:v>600</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="15">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="16">
                   <c:v>400</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="17">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="18">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="19">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="31">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="32">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="23">
+                <c:pt idx="33">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="24">
+                <c:pt idx="34">
                   <c:v>400</c:v>
                 </c:pt>
-                <c:pt idx="25">
+                <c:pt idx="35">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="26">
+                <c:pt idx="36">
                   <c:v>600</c:v>
                 </c:pt>
-                <c:pt idx="27">
+                <c:pt idx="37">
                   <c:v>700</c:v>
                 </c:pt>
-                <c:pt idx="28">
+                <c:pt idx="38">
                   <c:v>800</c:v>
                 </c:pt>
-                <c:pt idx="29">
+                <c:pt idx="39">
                   <c:v>900</c:v>
                 </c:pt>
-                <c:pt idx="30">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>1000</c:v>
-                </c:pt>
                 <c:pt idx="40">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="60">
                   <c:v>1000</c:v>
                 </c:pt>
               </c:numCache>
@@ -531,264 +672,384 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$42</c:f>
+              <c:f>Sheet1!$A$2:$A$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
+                <c:ptCount val="61"/>
                 <c:pt idx="0">
+                  <c:v>-400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-380</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-360</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-340</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-320</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-300</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-280</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-260</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-240</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-220</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>-200</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="11">
                   <c:v>-180</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="12">
                   <c:v>-160</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="13">
                   <c:v>-140</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="14">
                   <c:v>-120</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="15">
                   <c:v>-100</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="16">
                   <c:v>-80</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="17">
                   <c:v>-60</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="18">
                   <c:v>-40</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="19">
                   <c:v>-20</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="22">
                   <c:v>40</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="23">
                   <c:v>60</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="24">
                   <c:v>80</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="25">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="26">
                   <c:v>120</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="27">
                   <c:v>140</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="28">
                   <c:v>160</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="29">
                   <c:v>180</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="30">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="31">
                   <c:v>220</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="32">
                   <c:v>240</c:v>
                 </c:pt>
-                <c:pt idx="23">
+                <c:pt idx="33">
                   <c:v>260</c:v>
                 </c:pt>
-                <c:pt idx="24">
+                <c:pt idx="34">
                   <c:v>280</c:v>
                 </c:pt>
-                <c:pt idx="25">
+                <c:pt idx="35">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="26">
+                <c:pt idx="36">
                   <c:v>320</c:v>
                 </c:pt>
-                <c:pt idx="27">
+                <c:pt idx="37">
                   <c:v>340</c:v>
                 </c:pt>
-                <c:pt idx="28">
+                <c:pt idx="38">
                   <c:v>360</c:v>
                 </c:pt>
-                <c:pt idx="29">
+                <c:pt idx="39">
                   <c:v>380</c:v>
                 </c:pt>
-                <c:pt idx="30">
+                <c:pt idx="40">
                   <c:v>400</c:v>
                 </c:pt>
-                <c:pt idx="31">
+                <c:pt idx="41">
                   <c:v>420</c:v>
                 </c:pt>
-                <c:pt idx="32">
+                <c:pt idx="42">
                   <c:v>440</c:v>
                 </c:pt>
-                <c:pt idx="33">
+                <c:pt idx="43">
                   <c:v>460</c:v>
                 </c:pt>
-                <c:pt idx="34">
+                <c:pt idx="44">
                   <c:v>480</c:v>
                 </c:pt>
-                <c:pt idx="35">
+                <c:pt idx="45">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="36">
+                <c:pt idx="46">
                   <c:v>520</c:v>
                 </c:pt>
-                <c:pt idx="37">
+                <c:pt idx="47">
                   <c:v>540</c:v>
                 </c:pt>
-                <c:pt idx="38">
+                <c:pt idx="48">
                   <c:v>560</c:v>
                 </c:pt>
-                <c:pt idx="39">
+                <c:pt idx="49">
                   <c:v>580</c:v>
                 </c:pt>
-                <c:pt idx="40">
+                <c:pt idx="50">
                   <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>620</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>640</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>660</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>680</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>720</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>740</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>760</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>780</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>800</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$42</c:f>
+              <c:f>Sheet1!$C$2:$C$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
+                <c:ptCount val="61"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>900</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>800</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>700</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>600</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>400</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>300</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="22">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="23">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="24">
                   <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>700</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>800</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>900</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>1000</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>900</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>800</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>700</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>600</c:v>
                 </c:pt>
                 <c:pt idx="25">
                   <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="26">
+                  <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>800</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>800</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="36">
                   <c:v>400</c:v>
                 </c:pt>
-                <c:pt idx="27">
+                <c:pt idx="37">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="28">
+                <c:pt idx="38">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="29">
+                <c:pt idx="39">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="30">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="40">
                   <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>800</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>1000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -840,142 +1101,202 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$42</c:f>
+              <c:f>Sheet1!$A$2:$A$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
+                <c:ptCount val="61"/>
                 <c:pt idx="0">
+                  <c:v>-400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-380</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-360</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-340</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-320</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-300</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-280</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-260</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-240</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-220</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>-200</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="11">
                   <c:v>-180</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="12">
                   <c:v>-160</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="13">
                   <c:v>-140</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="14">
                   <c:v>-120</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="15">
                   <c:v>-100</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="16">
                   <c:v>-80</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="17">
                   <c:v>-60</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="18">
                   <c:v>-40</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="19">
                   <c:v>-20</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="22">
                   <c:v>40</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="23">
                   <c:v>60</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="24">
                   <c:v>80</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="25">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="26">
                   <c:v>120</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="27">
                   <c:v>140</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="28">
                   <c:v>160</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="29">
                   <c:v>180</c:v>
                 </c:pt>
-                <c:pt idx="20">
+                <c:pt idx="30">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="31">
                   <c:v>220</c:v>
                 </c:pt>
-                <c:pt idx="22">
+                <c:pt idx="32">
                   <c:v>240</c:v>
                 </c:pt>
-                <c:pt idx="23">
+                <c:pt idx="33">
                   <c:v>260</c:v>
                 </c:pt>
-                <c:pt idx="24">
+                <c:pt idx="34">
                   <c:v>280</c:v>
                 </c:pt>
-                <c:pt idx="25">
+                <c:pt idx="35">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="26">
+                <c:pt idx="36">
                   <c:v>320</c:v>
                 </c:pt>
-                <c:pt idx="27">
+                <c:pt idx="37">
                   <c:v>340</c:v>
                 </c:pt>
-                <c:pt idx="28">
+                <c:pt idx="38">
                   <c:v>360</c:v>
                 </c:pt>
-                <c:pt idx="29">
+                <c:pt idx="39">
                   <c:v>380</c:v>
                 </c:pt>
-                <c:pt idx="30">
+                <c:pt idx="40">
                   <c:v>400</c:v>
                 </c:pt>
-                <c:pt idx="31">
+                <c:pt idx="41">
                   <c:v>420</c:v>
                 </c:pt>
-                <c:pt idx="32">
+                <c:pt idx="42">
                   <c:v>440</c:v>
                 </c:pt>
-                <c:pt idx="33">
+                <c:pt idx="43">
                   <c:v>460</c:v>
                 </c:pt>
-                <c:pt idx="34">
+                <c:pt idx="44">
                   <c:v>480</c:v>
                 </c:pt>
-                <c:pt idx="35">
+                <c:pt idx="45">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="36">
+                <c:pt idx="46">
                   <c:v>520</c:v>
                 </c:pt>
-                <c:pt idx="37">
+                <c:pt idx="47">
                   <c:v>540</c:v>
                 </c:pt>
-                <c:pt idx="38">
+                <c:pt idx="48">
                   <c:v>560</c:v>
                 </c:pt>
-                <c:pt idx="39">
+                <c:pt idx="49">
                   <c:v>580</c:v>
                 </c:pt>
-                <c:pt idx="40">
+                <c:pt idx="50">
                   <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>620</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>640</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>660</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>680</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>720</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>740</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>760</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>780</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>800</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$42</c:f>
+              <c:f>Sheet1!$D$2:$D$62</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="41"/>
+                <c:ptCount val="61"/>
                 <c:pt idx="0">
                   <c:v>1000</c:v>
                 </c:pt>
@@ -1010,93 +1331,153 @@
                   <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="11">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="21">
                   <c:v>900</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="22">
                   <c:v>800</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="23">
                   <c:v>700</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="24">
                   <c:v>600</c:v>
                 </c:pt>
-                <c:pt idx="15">
+                <c:pt idx="25">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="16">
+                <c:pt idx="26">
                   <c:v>400</c:v>
                 </c:pt>
-                <c:pt idx="17">
+                <c:pt idx="27">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="18">
+                <c:pt idx="28">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="29">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="20">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="30">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="31">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="41">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="32">
+                <c:pt idx="42">
                   <c:v>200</c:v>
                 </c:pt>
-                <c:pt idx="33">
+                <c:pt idx="43">
                   <c:v>300</c:v>
                 </c:pt>
-                <c:pt idx="34">
+                <c:pt idx="44">
                   <c:v>400</c:v>
                 </c:pt>
-                <c:pt idx="35">
+                <c:pt idx="45">
                   <c:v>500</c:v>
                 </c:pt>
-                <c:pt idx="36">
+                <c:pt idx="46">
                   <c:v>600</c:v>
                 </c:pt>
-                <c:pt idx="37">
+                <c:pt idx="47">
                   <c:v>700</c:v>
                 </c:pt>
-                <c:pt idx="38">
+                <c:pt idx="48">
                   <c:v>800</c:v>
                 </c:pt>
-                <c:pt idx="39">
+                <c:pt idx="49">
                   <c:v>900</c:v>
                 </c:pt>
-                <c:pt idx="40">
+                <c:pt idx="50">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="60">
                   <c:v>1000</c:v>
                 </c:pt>
               </c:numCache>
@@ -1124,8 +1505,8 @@
         <c:axId val="1750441872"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="600"/>
-          <c:min val="-200"/>
+          <c:max val="800"/>
+          <c:min val="-400"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -1987,15 +2368,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2340,7 +2721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A8D5701-2811-4FC5-BA7F-0975CF01A108}">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="1" bestFit="1" customWidth="1"/>
@@ -2349,176 +2730,175 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6">
-        <v>-200</v>
-      </c>
-      <c r="B2" s="7">
-        <f>5*(-A2)</f>
-        <v>1000</v>
-      </c>
-      <c r="C2" s="6">
-        <v>0</v>
-      </c>
-      <c r="D2" s="9">
+        <v>-400</v>
+      </c>
+      <c r="B2" s="6">
+        <v>1000</v>
+      </c>
+      <c r="C2" s="8">
+        <v>1000</v>
+      </c>
+      <c r="D2" s="6">
         <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>-180</v>
-      </c>
-      <c r="B3" s="3">
-        <f t="shared" ref="B3:B12" si="0">5*(-A3)</f>
+        <v>-380</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C3" s="5">
+        <f t="shared" ref="C3:C10" si="0">-5*(A3+200)</f>
         <v>900</v>
       </c>
-      <c r="C3" s="1">
-        <v>0</v>
-      </c>
-      <c r="D3" s="4">
+      <c r="D3" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>-160</v>
-      </c>
-      <c r="B4" s="3">
+        <v>-360</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C4" s="5">
         <f t="shared" si="0"/>
         <v>800</v>
       </c>
-      <c r="C4" s="1">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4">
+      <c r="D4" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>-140</v>
-      </c>
-      <c r="B5" s="3">
+        <v>-340</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C5" s="5">
         <f t="shared" si="0"/>
         <v>700</v>
       </c>
-      <c r="C5" s="1">
-        <v>0</v>
-      </c>
-      <c r="D5" s="4">
+      <c r="D5" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>-120</v>
-      </c>
-      <c r="B6" s="3">
+        <v>-320</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C6" s="5">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
-      <c r="C6" s="1">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4">
+      <c r="D6" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>-100</v>
-      </c>
-      <c r="B7" s="3">
+        <v>-300</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C7" s="5">
         <f t="shared" si="0"/>
         <v>500</v>
       </c>
-      <c r="C7" s="1">
-        <v>0</v>
-      </c>
-      <c r="D7" s="4">
+      <c r="D7" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>-80</v>
-      </c>
-      <c r="B8" s="3">
+        <v>-280</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C8" s="5">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="C8" s="1">
-        <v>0</v>
-      </c>
-      <c r="D8" s="4">
+      <c r="D8" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>-60</v>
-      </c>
-      <c r="B9" s="3">
+        <v>-260</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C9" s="5">
         <f t="shared" si="0"/>
         <v>300</v>
       </c>
-      <c r="C9" s="1">
-        <v>0</v>
-      </c>
-      <c r="D9" s="4">
+      <c r="D9" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>-40</v>
-      </c>
-      <c r="B10" s="3">
+        <v>-240</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C10" s="5">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C10" s="1">
-        <v>0</v>
-      </c>
-      <c r="D10" s="4">
+      <c r="D10" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>-20</v>
-      </c>
-      <c r="B11" s="3">
-        <f t="shared" si="0"/>
+        <v>-220</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1000</v>
+      </c>
+      <c r="C11" s="5">
+        <f>-5*(A11+200)</f>
         <v>100</v>
       </c>
-      <c r="C11" s="1">
-        <v>0</v>
-      </c>
-      <c r="D11" s="4">
+      <c r="D11" s="1">
         <v>1000</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
-        <v>0</v>
+        <v>-200</v>
       </c>
       <c r="B12" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>5*(-A12)</f>
+        <v>1000</v>
       </c>
       <c r="C12" s="8">
         <v>0</v>
@@ -2529,470 +2909,770 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>20</v>
-      </c>
-      <c r="B13" s="1">
-        <v>0</v>
-      </c>
-      <c r="C13" s="5">
-        <f>A13*5</f>
-        <v>100</v>
+        <v>-180</v>
+      </c>
+      <c r="B13" s="3">
+        <f t="shared" ref="B13:B22" si="1">5*(-A13)</f>
+        <v>900</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0</v>
       </c>
       <c r="D13" s="4">
-        <f>5*(200-A13)</f>
-        <v>900</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>40</v>
-      </c>
-      <c r="B14" s="1">
-        <v>0</v>
-      </c>
-      <c r="C14" s="5">
-        <f t="shared" ref="C14:C22" si="1">A14*5</f>
-        <v>200</v>
+        <v>-160</v>
+      </c>
+      <c r="B14" s="3">
+        <f t="shared" si="1"/>
+        <v>800</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
       </c>
       <c r="D14" s="4">
-        <f t="shared" ref="D14:D22" si="2">5*(200-A14)</f>
-        <v>800</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>60</v>
-      </c>
-      <c r="B15" s="1">
-        <v>0</v>
-      </c>
-      <c r="C15" s="5">
+        <v>-140</v>
+      </c>
+      <c r="B15" s="3">
+        <f t="shared" si="1"/>
+        <v>700</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>-120</v>
+      </c>
+      <c r="B16" s="3">
+        <f t="shared" si="1"/>
+        <v>600</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>-100</v>
+      </c>
+      <c r="B17" s="3">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>-80</v>
+      </c>
+      <c r="B18" s="3">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+      <c r="C18" s="1">
+        <v>0</v>
+      </c>
+      <c r="D18" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>-60</v>
+      </c>
+      <c r="B19" s="3">
         <f t="shared" si="1"/>
         <v>300</v>
       </c>
-      <c r="D15" s="4">
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>-40</v>
+      </c>
+      <c r="B20" s="3">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>-20</v>
+      </c>
+      <c r="B21" s="3">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0</v>
+      </c>
+      <c r="D21" s="4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="6">
+        <v>0</v>
+      </c>
+      <c r="B22" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C22" s="8">
+        <v>0</v>
+      </c>
+      <c r="D22" s="9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>20</v>
+      </c>
+      <c r="B23" s="1">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5">
+        <f>A23*5</f>
+        <v>100</v>
+      </c>
+      <c r="D23" s="4">
+        <f>5*(200-A23)</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>40</v>
+      </c>
+      <c r="B24" s="1">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5">
+        <f t="shared" ref="C24:C32" si="2">A24*5</f>
+        <v>200</v>
+      </c>
+      <c r="D24" s="4">
+        <f t="shared" ref="D24:D32" si="3">5*(200-A24)</f>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>60</v>
+      </c>
+      <c r="B25" s="1">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="D25" s="4">
+        <f t="shared" si="3"/>
+        <v>700</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>80</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5">
+        <f t="shared" si="2"/>
+        <v>400</v>
+      </c>
+      <c r="D26" s="4">
+        <f t="shared" si="3"/>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>100</v>
+      </c>
+      <c r="B27" s="1">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="D27" s="4">
+        <f t="shared" si="3"/>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>120</v>
+      </c>
+      <c r="B28" s="1">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5">
+        <f t="shared" si="2"/>
+        <v>600</v>
+      </c>
+      <c r="D28" s="4">
+        <f t="shared" si="3"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>140</v>
+      </c>
+      <c r="B29" s="1">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5">
         <f t="shared" si="2"/>
         <v>700</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>80</v>
-      </c>
-      <c r="B16" s="1">
-        <v>0</v>
-      </c>
-      <c r="C16" s="5">
-        <f t="shared" si="1"/>
-        <v>400</v>
-      </c>
-      <c r="D16" s="4">
-        <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>100</v>
-      </c>
-      <c r="B17" s="1">
-        <v>0</v>
-      </c>
-      <c r="C17" s="5">
-        <f t="shared" si="1"/>
-        <v>500</v>
-      </c>
-      <c r="D17" s="4">
-        <f t="shared" si="2"/>
-        <v>500</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>120</v>
-      </c>
-      <c r="B18" s="1">
-        <v>0</v>
-      </c>
-      <c r="C18" s="5">
-        <f t="shared" si="1"/>
-        <v>600</v>
-      </c>
-      <c r="D18" s="4">
-        <f t="shared" si="2"/>
-        <v>400</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>140</v>
-      </c>
-      <c r="B19" s="1">
-        <v>0</v>
-      </c>
-      <c r="C19" s="5">
-        <f t="shared" si="1"/>
-        <v>700</v>
-      </c>
-      <c r="D19" s="4">
-        <f t="shared" si="2"/>
-        <v>300</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>160</v>
-      </c>
-      <c r="B20" s="1">
-        <v>0</v>
-      </c>
-      <c r="C20" s="5">
-        <f t="shared" si="1"/>
-        <v>800</v>
-      </c>
-      <c r="D20" s="4">
-        <f t="shared" si="2"/>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>180</v>
-      </c>
-      <c r="B21" s="1">
-        <v>0</v>
-      </c>
-      <c r="C21" s="5">
-        <f t="shared" si="1"/>
-        <v>900</v>
-      </c>
-      <c r="D21" s="4">
-        <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
-        <v>200</v>
-      </c>
-      <c r="B22" s="7">
-        <v>0</v>
-      </c>
-      <c r="C22" s="8">
-        <f t="shared" si="1"/>
-        <v>1000</v>
-      </c>
-      <c r="D22" s="9">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>220</v>
-      </c>
-      <c r="B23" s="3">
-        <f>5*(A23-200)</f>
-        <v>100</v>
-      </c>
-      <c r="C23" s="5">
-        <f>5*(400-A23)</f>
-        <v>900</v>
-      </c>
-      <c r="D23" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>240</v>
-      </c>
-      <c r="B24" s="3">
-        <f t="shared" ref="B24:B31" si="3">5*(A24-200)</f>
-        <v>200</v>
-      </c>
-      <c r="C24" s="5">
-        <f t="shared" ref="C24:C32" si="4">5*(400-A24)</f>
-        <v>800</v>
-      </c>
-      <c r="D24" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>260</v>
-      </c>
-      <c r="B25" s="3">
+      <c r="D29" s="4">
         <f t="shared" si="3"/>
         <v>300</v>
       </c>
-      <c r="C25" s="5">
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>160</v>
+      </c>
+      <c r="B30" s="1">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5">
+        <f t="shared" si="2"/>
+        <v>800</v>
+      </c>
+      <c r="D30" s="4">
+        <f t="shared" si="3"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>180</v>
+      </c>
+      <c r="B31" s="1">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5">
+        <f t="shared" si="2"/>
+        <v>900</v>
+      </c>
+      <c r="D31" s="4">
+        <f t="shared" si="3"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="6">
+        <v>200</v>
+      </c>
+      <c r="B32" s="7">
+        <v>0</v>
+      </c>
+      <c r="C32" s="8">
+        <f t="shared" si="2"/>
+        <v>1000</v>
+      </c>
+      <c r="D32" s="9">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>220</v>
+      </c>
+      <c r="B33" s="3">
+        <f>5*(A33-200)</f>
+        <v>100</v>
+      </c>
+      <c r="C33" s="5">
+        <f>5*(400-A33)</f>
+        <v>900</v>
+      </c>
+      <c r="D33" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>240</v>
+      </c>
+      <c r="B34" s="3">
+        <f t="shared" ref="B34:B41" si="4">5*(A34-200)</f>
+        <v>200</v>
+      </c>
+      <c r="C34" s="5">
+        <f t="shared" ref="C34:C42" si="5">5*(400-A34)</f>
+        <v>800</v>
+      </c>
+      <c r="D34" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>260</v>
+      </c>
+      <c r="B35" s="3">
+        <f t="shared" si="4"/>
+        <v>300</v>
+      </c>
+      <c r="C35" s="5">
+        <f t="shared" si="5"/>
+        <v>700</v>
+      </c>
+      <c r="D35" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>280</v>
+      </c>
+      <c r="B36" s="3">
+        <f t="shared" si="4"/>
+        <v>400</v>
+      </c>
+      <c r="C36" s="5">
+        <f t="shared" si="5"/>
+        <v>600</v>
+      </c>
+      <c r="D36" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>300</v>
+      </c>
+      <c r="B37" s="3">
+        <f t="shared" si="4"/>
+        <v>500</v>
+      </c>
+      <c r="C37" s="5">
+        <f t="shared" si="5"/>
+        <v>500</v>
+      </c>
+      <c r="D37" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>320</v>
+      </c>
+      <c r="B38" s="3">
+        <f t="shared" si="4"/>
+        <v>600</v>
+      </c>
+      <c r="C38" s="5">
+        <f t="shared" si="5"/>
+        <v>400</v>
+      </c>
+      <c r="D38" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>340</v>
+      </c>
+      <c r="B39" s="3">
         <f t="shared" si="4"/>
         <v>700</v>
       </c>
-      <c r="D25" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>280</v>
-      </c>
-      <c r="B26" s="3">
-        <f t="shared" si="3"/>
-        <v>400</v>
-      </c>
-      <c r="C26" s="5">
-        <f t="shared" si="4"/>
-        <v>600</v>
-      </c>
-      <c r="D26" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>300</v>
-      </c>
-      <c r="B27" s="3">
-        <f t="shared" si="3"/>
-        <v>500</v>
-      </c>
-      <c r="C27" s="5">
-        <f t="shared" si="4"/>
-        <v>500</v>
-      </c>
-      <c r="D27" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <v>320</v>
-      </c>
-      <c r="B28" s="3">
-        <f t="shared" si="3"/>
-        <v>600</v>
-      </c>
-      <c r="C28" s="5">
-        <f t="shared" si="4"/>
-        <v>400</v>
-      </c>
-      <c r="D28" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <v>340</v>
-      </c>
-      <c r="B29" s="3">
-        <f t="shared" si="3"/>
-        <v>700</v>
-      </c>
-      <c r="C29" s="5">
-        <f t="shared" si="4"/>
-        <v>300</v>
-      </c>
-      <c r="D29" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
-        <v>360</v>
-      </c>
-      <c r="B30" s="3">
-        <f t="shared" si="3"/>
-        <v>800</v>
-      </c>
-      <c r="C30" s="5">
-        <f t="shared" si="4"/>
-        <v>200</v>
-      </c>
-      <c r="D30" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
-        <v>380</v>
-      </c>
-      <c r="B31" s="3">
-        <f t="shared" si="3"/>
-        <v>900</v>
-      </c>
-      <c r="C31" s="5">
-        <f t="shared" si="4"/>
-        <v>100</v>
-      </c>
-      <c r="D31" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="6">
-        <v>400</v>
-      </c>
-      <c r="B32" s="7">
-        <v>1000</v>
-      </c>
-      <c r="C32" s="8">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="D32" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
-        <v>420</v>
-      </c>
-      <c r="B33" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C33" s="1">
-        <v>0</v>
-      </c>
-      <c r="D33" s="4">
-        <f>5*(A33-400)</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
-        <v>440</v>
-      </c>
-      <c r="B34" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C34" s="1">
-        <v>0</v>
-      </c>
-      <c r="D34" s="4">
-        <f t="shared" ref="D34:D42" si="5">5*(A34-400)</f>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>460</v>
-      </c>
-      <c r="B35" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C35" s="1">
-        <v>0</v>
-      </c>
-      <c r="D35" s="4">
+      <c r="C39" s="5">
         <f t="shared" si="5"/>
         <v>300</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <v>480</v>
-      </c>
-      <c r="B36" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C36" s="1">
-        <v>0</v>
-      </c>
-      <c r="D36" s="4">
-        <f t="shared" si="5"/>
-        <v>400</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
-        <v>500</v>
-      </c>
-      <c r="B37" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C37" s="1">
-        <v>0</v>
-      </c>
-      <c r="D37" s="4">
-        <f t="shared" si="5"/>
-        <v>500</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <v>520</v>
-      </c>
-      <c r="B38" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C38" s="1">
-        <v>0</v>
-      </c>
-      <c r="D38" s="4">
-        <f t="shared" si="5"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
-        <v>540</v>
-      </c>
-      <c r="B39" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C39" s="1">
-        <v>0</v>
-      </c>
-      <c r="D39" s="4">
-        <f t="shared" si="5"/>
-        <v>700</v>
+      <c r="D39" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>560</v>
+        <v>360</v>
       </c>
       <c r="B40" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C40" s="1">
-        <v>0</v>
-      </c>
-      <c r="D40" s="4">
+        <f t="shared" si="4"/>
+        <v>800</v>
+      </c>
+      <c r="C40" s="5">
         <f t="shared" si="5"/>
-        <v>800</v>
+        <v>200</v>
+      </c>
+      <c r="D40" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>580</v>
+        <v>380</v>
       </c>
       <c r="B41" s="3">
-        <v>1000</v>
-      </c>
-      <c r="C41" s="1">
-        <v>0</v>
-      </c>
-      <c r="D41" s="4">
+        <f t="shared" si="4"/>
+        <v>900</v>
+      </c>
+      <c r="C41" s="5">
         <f t="shared" si="5"/>
-        <v>900</v>
+        <v>100</v>
+      </c>
+      <c r="D41" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="6">
+        <v>400</v>
+      </c>
+      <c r="B42" s="7">
+        <v>1000</v>
+      </c>
+      <c r="C42" s="8">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="D42" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>420</v>
+      </c>
+      <c r="B43" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C43" s="1">
+        <v>0</v>
+      </c>
+      <c r="D43" s="4">
+        <f>5*(A43-400)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>440</v>
+      </c>
+      <c r="B44" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C44" s="1">
+        <v>0</v>
+      </c>
+      <c r="D44" s="4">
+        <f t="shared" ref="D44:D62" si="6">5*(A44-400)</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>460</v>
+      </c>
+      <c r="B45" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C45" s="1">
+        <v>0</v>
+      </c>
+      <c r="D45" s="4">
+        <f t="shared" si="6"/>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>480</v>
+      </c>
+      <c r="B46" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C46" s="1">
+        <v>0</v>
+      </c>
+      <c r="D46" s="4">
+        <f t="shared" si="6"/>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>500</v>
+      </c>
+      <c r="B47" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C47" s="1">
+        <v>0</v>
+      </c>
+      <c r="D47" s="4">
+        <f t="shared" si="6"/>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>520</v>
+      </c>
+      <c r="B48" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C48" s="1">
+        <v>0</v>
+      </c>
+      <c r="D48" s="4">
+        <f t="shared" si="6"/>
         <v>600</v>
       </c>
-      <c r="B42" s="7">
-        <v>1000</v>
-      </c>
-      <c r="C42" s="6">
-        <v>0</v>
-      </c>
-      <c r="D42" s="9">
-        <f t="shared" si="5"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>540</v>
+      </c>
+      <c r="B49" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C49" s="1">
+        <v>0</v>
+      </c>
+      <c r="D49" s="4">
+        <f t="shared" si="6"/>
+        <v>700</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>560</v>
+      </c>
+      <c r="B50" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C50" s="1">
+        <v>0</v>
+      </c>
+      <c r="D50" s="4">
+        <f t="shared" si="6"/>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>580</v>
+      </c>
+      <c r="B51" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0</v>
+      </c>
+      <c r="D51" s="4">
+        <f t="shared" si="6"/>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="6">
+        <v>600</v>
+      </c>
+      <c r="B52" s="11">
+        <v>1000</v>
+      </c>
+      <c r="C52" s="8">
+        <v>0</v>
+      </c>
+      <c r="D52" s="9">
+        <f t="shared" si="6"/>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>620</v>
+      </c>
+      <c r="B53" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C53" s="5">
+        <f>5*(A53-600)</f>
+        <v>100</v>
+      </c>
+      <c r="D53" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>640</v>
+      </c>
+      <c r="B54" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C54" s="5">
+        <f t="shared" ref="C54:C62" si="7">5*(A54-600)</f>
+        <v>200</v>
+      </c>
+      <c r="D54" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>660</v>
+      </c>
+      <c r="B55" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C55" s="5">
+        <f t="shared" si="7"/>
+        <v>300</v>
+      </c>
+      <c r="D55" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>680</v>
+      </c>
+      <c r="B56" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C56" s="5">
+        <f t="shared" si="7"/>
+        <v>400</v>
+      </c>
+      <c r="D56" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>700</v>
+      </c>
+      <c r="B57" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C57" s="5">
+        <f t="shared" si="7"/>
+        <v>500</v>
+      </c>
+      <c r="D57" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>720</v>
+      </c>
+      <c r="B58" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C58" s="5">
+        <f t="shared" si="7"/>
+        <v>600</v>
+      </c>
+      <c r="D58" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>740</v>
+      </c>
+      <c r="B59" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C59" s="5">
+        <f t="shared" si="7"/>
+        <v>700</v>
+      </c>
+      <c r="D59" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>760</v>
+      </c>
+      <c r="B60" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C60" s="5">
+        <f t="shared" si="7"/>
+        <v>800</v>
+      </c>
+      <c r="D60" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>780</v>
+      </c>
+      <c r="B61" s="10">
+        <v>1000</v>
+      </c>
+      <c r="C61" s="5">
+        <f t="shared" si="7"/>
+        <v>900</v>
+      </c>
+      <c r="D61" s="1">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="6">
+        <v>800</v>
+      </c>
+      <c r="B62" s="11">
+        <v>1000</v>
+      </c>
+      <c r="C62" s="8">
+        <f t="shared" si="7"/>
+        <v>1000</v>
+      </c>
+      <c r="D62" s="6">
         <v>1000</v>
       </c>
     </row>

</xml_diff>